<commit_message>
CRM locked to light brand theme; journey test report and screenshots; workbook update
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q1YFQVkqvZuZSxHETxCkHf
</commit_message>
<xml_diff>
--- a/business/knock-unit-economics.xlsx
+++ b/business/knock-unit-economics.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="86">
   <si>
     <t xml:space="preserve">Cost, price and margin per client: change the yellow cells here and on Inputs</t>
   </si>
@@ -81,13 +81,10 @@
     <t xml:space="preserve">Full, 21 days</t>
   </si>
   <si>
-    <t xml:space="preserve">Done-for-you (founding)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Done-for-you (standard)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Notes: Claude cost uses the step assumptions on Inputs (estimates until measured with the cost command). Done-for-you tool cost = one La Growth Machine Basic identity month (about $70). Founder hours are estimates.</t>
+    <t xml:space="preserve">Done-for-you (later, not offered now)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Notes: Claude cost uses the step assumptions on Inputs (estimates until measured with the cost command). Done-for-you tool cost = one La Growth Machine Basic identity month (about $70). Founder hours = support and spot checks only (automation runs as scheduled Claude Code tasks; the client approves and sends).</t>
   </si>
   <si>
     <t xml:space="preserve">Knock unit economics: change the yellow cells</t>
@@ -752,7 +749,7 @@
         <v>60</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E4" s="3" t="n">
         <v>0</v>
@@ -779,19 +776,19 @@
       </c>
       <c r="K4" s="4" t="n">
         <f aca="false">D4*Inputs!$B$8</f>
-        <v>2500</v>
+        <v>250</v>
       </c>
       <c r="L4" s="4" t="n">
         <f aca="false">SUM(E4:K4)</f>
-        <v>4078.6148</v>
+        <v>1828.6148</v>
       </c>
       <c r="M4" s="4" t="n">
         <f aca="false">B4-L4</f>
-        <v>-1579.6148</v>
+        <v>670.3852</v>
       </c>
       <c r="N4" s="5" t="n">
         <f aca="false">M4/B4</f>
-        <v>-0.632098759503802</v>
+        <v>0.268261384553822</v>
       </c>
       <c r="O4" s="5" t="n">
         <f aca="false">(M4+K4)/B4</f>
@@ -809,7 +806,7 @@
         <v>120</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>8</v>
+        <v>0.75</v>
       </c>
       <c r="E5" s="3" t="n">
         <v>0</v>
@@ -836,19 +833,19 @@
       </c>
       <c r="K5" s="4" t="n">
         <f aca="false">D5*Inputs!$B$8</f>
-        <v>4000</v>
+        <v>375</v>
       </c>
       <c r="L5" s="4" t="n">
         <f aca="false">SUM(E5:K5)</f>
-        <v>6589.6532</v>
+        <v>2964.6532</v>
       </c>
       <c r="M5" s="4" t="n">
         <f aca="false">B5-L5</f>
-        <v>-2590.6532</v>
+        <v>1034.3468</v>
       </c>
       <c r="N5" s="5" t="n">
         <f aca="false">M5/B5</f>
-        <v>-0.647825256314079</v>
+        <v>0.25865136284071</v>
       </c>
       <c r="O5" s="5" t="n">
         <f aca="false">(M5+K5)/B5</f>
@@ -866,7 +863,7 @@
         <v>180</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="E6" s="3" t="n">
         <v>0</v>
@@ -893,19 +890,19 @@
       </c>
       <c r="K6" s="4" t="n">
         <f aca="false">D6*Inputs!$B$8</f>
-        <v>5500</v>
+        <v>500</v>
       </c>
       <c r="L6" s="4" t="n">
         <f aca="false">SUM(E6:K6)</f>
-        <v>9100.6916</v>
+        <v>4100.6916</v>
       </c>
       <c r="M6" s="4" t="n">
         <f aca="false">B6-L6</f>
-        <v>-3601.6916</v>
+        <v>1398.3084</v>
       </c>
       <c r="N6" s="5" t="n">
         <f aca="false">M6/B6</f>
-        <v>-0.654972104018913</v>
+        <v>0.254284124386252</v>
       </c>
       <c r="O6" s="5" t="n">
         <f aca="false">(M6+K6)/B6</f>
@@ -917,7 +914,7 @@
         <v>19</v>
       </c>
       <c r="B7" s="3" t="n">
-        <v>14999</v>
+        <v>19999</v>
       </c>
       <c r="C7" s="3" t="n">
         <v>180</v>
@@ -938,7 +935,7 @@
       </c>
       <c r="H7" s="4" t="n">
         <f aca="false">B7*Inputs!$B$5</f>
-        <v>353.9764</v>
+        <v>471.9764</v>
       </c>
       <c r="I7" s="4" t="n">
         <f aca="false">B7-B7/(1+Inputs!$B$7*Inputs!$B$6)</f>
@@ -954,81 +951,24 @@
       </c>
       <c r="L7" s="4" t="n">
         <f aca="false">SUM(E7:K7)</f>
-        <v>17984.8916</v>
+        <v>18102.8916</v>
       </c>
       <c r="M7" s="4" t="n">
         <f aca="false">B7-L7</f>
-        <v>-2985.8916</v>
+        <v>1896.1084</v>
       </c>
       <c r="N7" s="5" t="n">
         <f aca="false">M7/B7</f>
-        <v>-0.199072711514101</v>
+        <v>0.0948101605080253</v>
       </c>
       <c r="O7" s="5" t="n">
         <f aca="false">(M7+K7)/B7</f>
-        <v>0.334296179745316</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
-        <v>20</v>
-      </c>
-      <c r="B8" s="3" t="n">
-        <v>19999</v>
-      </c>
-      <c r="C8" s="3" t="n">
-        <v>180</v>
-      </c>
-      <c r="D8" s="3" t="n">
-        <v>16</v>
-      </c>
-      <c r="E8" s="3" t="n">
-        <v>6160</v>
-      </c>
-      <c r="F8" s="4" t="n">
-        <f aca="false">C8*'Cost per prospect'!$C$13</f>
-        <v>2926.9152</v>
-      </c>
-      <c r="G8" s="4" t="n">
-        <f aca="false">Inputs!$B$49*Inputs!$B$4</f>
-        <v>44</v>
-      </c>
-      <c r="H8" s="4" t="n">
-        <f aca="false">B8*Inputs!$B$5</f>
-        <v>471.9764</v>
-      </c>
-      <c r="I8" s="4" t="n">
-        <f aca="false">B8-B8/(1+Inputs!$B$7*Inputs!$B$6)</f>
-        <v>0</v>
-      </c>
-      <c r="J8" s="4" t="n">
-        <f aca="false">Inputs!$B$9/Inputs!$B$10</f>
-        <v>500</v>
-      </c>
-      <c r="K8" s="4" t="n">
-        <f aca="false">D8*Inputs!$B$8</f>
-        <v>8000</v>
-      </c>
-      <c r="L8" s="4" t="n">
-        <f aca="false">SUM(E8:K8)</f>
-        <v>18102.8916</v>
-      </c>
-      <c r="M8" s="4" t="n">
-        <f aca="false">B8-L8</f>
-        <v>1896.1084</v>
-      </c>
-      <c r="N8" s="5" t="n">
-        <f aca="false">M8/B8</f>
-        <v>0.0948101605080253</v>
-      </c>
-      <c r="O8" s="5" t="n">
-        <f aca="false">(M8+K8)/B8</f>
         <v>0.494830161508075</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -1057,17 +997,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B4" s="3" t="n">
         <v>88</v>
@@ -1075,7 +1015,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B5" s="3" t="n">
         <v>0.0236</v>
@@ -1083,7 +1023,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B6" s="3" t="n">
         <v>0</v>
@@ -1091,7 +1031,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B7" s="3" t="n">
         <v>0.18</v>
@@ -1099,18 +1039,18 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B8" s="3" t="n">
         <v>500</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B9" s="3" t="n">
         <v>2500</v>
@@ -1118,7 +1058,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B10" s="3" t="n">
         <v>5</v>
@@ -1126,12 +1066,12 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B12" s="3" t="n">
         <v>4</v>
@@ -1139,7 +1079,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B13" s="3" t="n">
         <v>20</v>
@@ -1147,7 +1087,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B14" s="3" t="n">
         <v>2</v>
@@ -1155,7 +1095,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B15" s="3" t="n">
         <v>10</v>
@@ -1163,7 +1103,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B16" s="3" t="n">
         <v>1</v>
@@ -1171,7 +1111,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="0" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B17" s="3" t="n">
         <v>5</v>
@@ -1179,7 +1119,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="0" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B18" s="3" t="n">
         <v>0.01</v>
@@ -1187,23 +1127,23 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="0" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B19" s="3" t="n">
         <v>0.3</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="0" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B21" s="3" t="n">
         <v>2000</v>
@@ -1211,7 +1151,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="0" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B22" s="3" t="n">
         <v>300</v>
@@ -1219,7 +1159,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="0" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B23" s="3" t="n">
         <v>3</v>
@@ -1227,7 +1167,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="0" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B24" s="3" t="n">
         <v>2</v>
@@ -1235,7 +1175,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="0" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B25" s="3" t="n">
         <v>6000</v>
@@ -1243,7 +1183,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="0" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B26" s="3" t="n">
         <v>800</v>
@@ -1251,7 +1191,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="0" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B27" s="3" t="n">
         <v>2</v>
@@ -1259,7 +1199,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="0" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B28" s="3" t="n">
         <v>6000</v>
@@ -1267,7 +1207,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="0" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B29" s="3" t="n">
         <v>1500</v>
@@ -1275,7 +1215,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="0" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B30" s="3" t="n">
         <v>1</v>
@@ -1283,7 +1223,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="0" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B31" s="3" t="n">
         <v>3</v>
@@ -1291,7 +1231,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="0" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B32" s="3" t="n">
         <v>3000</v>
@@ -1299,7 +1239,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="0" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B33" s="3" t="n">
         <v>600</v>
@@ -1307,7 +1247,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="0" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B34" s="3" t="n">
         <v>2</v>
@@ -1315,7 +1255,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="0" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B35" s="3" t="n">
         <v>4000</v>
@@ -1323,7 +1263,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="0" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B36" s="3" t="n">
         <v>800</v>
@@ -1331,7 +1271,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="0" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B37" s="3" t="n">
         <v>1</v>
@@ -1339,7 +1279,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="0" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B38" s="3" t="n">
         <v>1</v>
@@ -1347,12 +1287,12 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="6" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="0" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B40" s="3" t="n">
         <v>0.7</v>
@@ -1360,7 +1300,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="0" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B41" s="3" t="n">
         <v>3000</v>
@@ -1368,7 +1308,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="0" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B42" s="3" t="n">
         <v>500</v>
@@ -1376,7 +1316,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="0" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B43" s="3" t="n">
         <v>1</v>
@@ -1384,18 +1324,18 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="0" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B44" s="3" t="n">
         <v>0.3</v>
       </c>
       <c r="C44" s="7" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="0" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B45" s="3" t="n">
         <v>2</v>
@@ -1403,7 +1343,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="0" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B46" s="3" t="n">
         <v>5000</v>
@@ -1411,7 +1351,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="0" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B47" s="3" t="n">
         <v>800</v>
@@ -1419,7 +1359,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="0" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B48" s="3" t="n">
         <v>1</v>
@@ -1427,7 +1367,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="0" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B49" s="3" t="n">
         <v>0.5</v>
@@ -1458,23 +1398,23 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="B3" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="C3" s="6" t="s">
         <v>75</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B4" s="8" t="n">
         <f aca="false">(1)*(Inputs!$B$21*CHOOSE(Inputs!$B$23,Inputs!$B$12,Inputs!$B$14,Inputs!$B$16)*(1-Inputs!$B$19)+Inputs!$B$22*CHOOSE(Inputs!$B$23,Inputs!$B$13,Inputs!$B$15,Inputs!$B$17))/1000000</f>
@@ -1487,7 +1427,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B5" s="8" t="n">
         <f aca="false">(1)*(Inputs!$B$25*CHOOSE(Inputs!$B$27,Inputs!$B$12,Inputs!$B$14,Inputs!$B$16)*(1-Inputs!$B$19)+Inputs!$B$26*CHOOSE(Inputs!$B$27,Inputs!$B$13,Inputs!$B$15,Inputs!$B$17))/1000000</f>
@@ -1500,7 +1440,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B6" s="8" t="n">
         <f aca="false">Inputs!$B$24*Inputs!$B$18</f>
@@ -1513,7 +1453,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B7" s="8" t="n">
         <f aca="false">Inputs!$B$38*Inputs!$B$18</f>
@@ -1526,7 +1466,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B8" s="8" t="n">
         <f aca="false">(1)*(Inputs!$B$28*CHOOSE(Inputs!$B$30,Inputs!$B$12,Inputs!$B$14,Inputs!$B$16)*(1-Inputs!$B$19)+Inputs!$B$29*CHOOSE(Inputs!$B$30,Inputs!$B$13,Inputs!$B$15,Inputs!$B$17))/1000000</f>
@@ -1539,7 +1479,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B9" s="8" t="n">
         <f aca="false">(Inputs!$B$31)*(Inputs!$B$32*CHOOSE(Inputs!$B$34,Inputs!$B$12,Inputs!$B$14,Inputs!$B$16)*(1-Inputs!$B$19)+Inputs!$B$33*CHOOSE(Inputs!$B$34,Inputs!$B$13,Inputs!$B$15,Inputs!$B$17))/1000000</f>
@@ -1552,7 +1492,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B10" s="8" t="n">
         <f aca="false">(1)*(Inputs!$B$35*CHOOSE(Inputs!$B$37,Inputs!$B$12,Inputs!$B$14,Inputs!$B$16)*(1-Inputs!$B$19)+Inputs!$B$36*CHOOSE(Inputs!$B$37,Inputs!$B$13,Inputs!$B$15,Inputs!$B$17))/1000000</f>
@@ -1565,7 +1505,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B11" s="8" t="n">
         <f aca="false">(Inputs!$B$40)*(Inputs!$B$41*CHOOSE(Inputs!$B$43,Inputs!$B$12,Inputs!$B$14,Inputs!$B$16)*(1-Inputs!$B$19)+Inputs!$B$42*CHOOSE(Inputs!$B$43,Inputs!$B$13,Inputs!$B$15,Inputs!$B$17))/1000000</f>
@@ -1578,7 +1518,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B12" s="8" t="n">
         <f aca="false">(Inputs!$B$44*Inputs!$B$45)*(Inputs!$B$46*CHOOSE(Inputs!$B$48,Inputs!$B$12,Inputs!$B$14,Inputs!$B$16)*(1-Inputs!$B$19)+Inputs!$B$47*CHOOSE(Inputs!$B$48,Inputs!$B$13,Inputs!$B$15,Inputs!$B$17))/1000000</f>
@@ -1591,7 +1531,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B13" s="8" t="n">
         <f aca="false">SUM(B4:B12)</f>

</xml_diff>